<commit_message>
ultimo commit antes de formatar
</commit_message>
<xml_diff>
--- a/banco_de_dados/caderno_anotacoes.xlsx
+++ b/banco_de_dados/caderno_anotacoes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -587,90 +587,6 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>Tirar duvidas sobre essa questão se possível, a se sentar não seria o equivalente a sentando? se sim essa frase também é ambígua</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>29</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>31/12/2025 11:55</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>225</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Português</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Regência Verbal</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>O verbo “querer”, no sentido de “estimar”/“querer bem a”, é VTI e exige a preposição “a”</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>31</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>31/12/2025 12:12</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>222</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Português</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Regência Verbal</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Como assim verbo VTI exige preposição?</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>32</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>09/01/2026 10:57</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>1810</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Conhecimentos Específicos</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Logística</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Criar flashcards para o conteúdo de logística da transpetro</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
:up: algumas questoes respondidas
</commit_message>
<xml_diff>
--- a/banco_de_dados/caderno_anotacoes.xlsx
+++ b/banco_de_dados/caderno_anotacoes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -587,6 +587,34 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>Tirar duvidas sobre essa questão se possível, a se sentar não seria o equivalente a sentando? se sim essa frase também é ambígua</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>29</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>28/03/2026 23:21</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1971</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Diagramas Lógicos</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Não entendi esse comentário. Na questão fala que todos os que gostam de futebol também gostam de voleibol, mas não fala nada sobre todos os que gostam de voleibol também gostarem de futebol. Poderiam existir os que gostam de voleibol mas não gostam de futebol</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
:up: algumas questões respondidas
</commit_message>
<xml_diff>
--- a/banco_de_dados/caderno_anotacoes.xlsx
+++ b/banco_de_dados/caderno_anotacoes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -618,6 +618,34 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>30</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>08/04/2026 03:48</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>812</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Pesquisa Operacional</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Mais atenção na leitura "90% NUNCA foram assaltadas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: algumas questões cadastradas - RL
</commit_message>
<xml_diff>
--- a/banco_de_dados/caderno_anotacoes.xlsx
+++ b/banco_de_dados/caderno_anotacoes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -646,6 +646,34 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>31</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>10/04/2026 08:39</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1340</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Equivalência de Capitais</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Aprender a fórmula do Valor Presente (VP)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: algumas questões respondidas = CE
</commit_message>
<xml_diff>
--- a/banco_de_dados/caderno_anotacoes.xlsx
+++ b/banco_de_dados/caderno_anotacoes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -674,6 +674,34 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>33</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>10/04/2026 15:31</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>868</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Gestão de Estoques</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Atenção às unidades de media, mensal/semanal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: alguns flashcards criados
</commit_message>
<xml_diff>
--- a/banco_de_dados/caderno_anotacoes.xlsx
+++ b/banco_de_dados/caderno_anotacoes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -702,6 +702,122 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>34</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>11/04/2026 09:09</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>670</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Ver essa questão depois</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>35</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>11/04/2026 09:10</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>678</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Ver esse PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>36</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>11/04/2026 09:38</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2611</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Gestão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Pesquisar sobre esses princípios básicos da teoria da atividade</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>37</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>11/04/2026 09:43</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2609</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Gestão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Buscar os autores que sustentam essa tese</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: algumas questões respondidas - portugues
</commit_message>
<xml_diff>
--- a/banco_de_dados/caderno_anotacoes.xlsx
+++ b/banco_de_dados/caderno_anotacoes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -846,6 +846,90 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>39</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>14/04/2026 09:50</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>129</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Funções Sintáticas</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>verificar o desempenho nessa questão (respostas anteriores)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>40</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>14/04/2026 09:54</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>130</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Funções Sintáticas</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>criar um cadr sobre as diferenças entre adjunto adnominal de complemento nominal</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>41</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>14/04/2026 10:13</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>135</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Funções Sintáticas</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>mas uma vez errando por não se atentar palavra "Incorreta"</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: algumas questoes respondidas - port
</commit_message>
<xml_diff>
--- a/banco_de_dados/caderno_anotacoes.xlsx
+++ b/banco_de_dados/caderno_anotacoes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -930,6 +930,90 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>42</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>18/08/2026 16:19</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>300</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Mecanismos de Coesão Textual</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>cria resumo dessa questão</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>43</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>18/08/2026 21:28</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>66</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Morfologia</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>fazer resumo dessa questão</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>44</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>18/08/2026 21:31</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>52</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Morfologia</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>fazer um resumo desta</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: algumas questoes respondidas - mat
</commit_message>
<xml_diff>
--- a/banco_de_dados/caderno_anotacoes.xlsx
+++ b/banco_de_dados/caderno_anotacoes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1186,6 +1186,90 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>51</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>19/08/2026 11:23</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>4515</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Análise Combinatória</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>resumo e comentários dessa questão</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>52</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>19/08/2026 11:40</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>2038</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Análise Combinatória</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>rever se essa questão pode ser feita por arranjo como eu fiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>53</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>19/08/2026 11:46</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>3893</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Conjuntos Numéricos</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>ridícula</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: algumas questoes respondiddas, mat
</commit_message>
<xml_diff>
--- a/banco_de_dados/caderno_anotacoes.xlsx
+++ b/banco_de_dados/caderno_anotacoes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1270,6 +1270,119 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>54</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>21/08/2026 11:18</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>4303</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Geometria Espacial</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fazer resumo de circunscrição de sólidos, acertei no chute
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>55</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>21/08/2026 11:21</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>4281</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Geometria Espacial</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>fazer um resumo sobre fórmulas geométricas de um tetraedro, acertei no chute</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>56</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>21/08/2026 11:26</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>4299</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Geometria Espacial</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>fazer um resumo sobre fórmulas geométricas de um cone</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>57</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>21/08/2026 23:31</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>4283</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Geometria Espacial</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>fazer um resumo sobre as formulas das figuras geometricas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>